<commit_message>
Updated EW-Systems and Mech-Weapons documentation
</commit_message>
<xml_diff>
--- a/docs/Mech-Weapons.xlsx
+++ b/docs/Mech-Weapons.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FoundryData-Dev\Data\systems\mwd\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Apps\MWD-main\MWD\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FD2ABD-81A4-4D60-AA8F-6E01C5389A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71EB75E-FE7B-4A01-9A69-63729643ACF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{E1E4146D-AA47-4F02-8EE5-13D857F0DD65}"/>
+    <workbookView xWindow="5760" yWindow="1740" windowWidth="38700" windowHeight="15345" xr2:uid="{E1E4146D-AA47-4F02-8EE5-13D857F0DD65}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="106">
   <si>
     <t>Weapon</t>
   </si>
@@ -295,6 +295,66 @@
   </si>
   <si>
     <t>6</t>
+  </si>
+  <si>
+    <t>Tonnage/10</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>Pilot REF</t>
+  </si>
+  <si>
+    <t>Sword</t>
+  </si>
+  <si>
+    <t>Axe</t>
+  </si>
+  <si>
+    <t>Katana</t>
+  </si>
+  <si>
+    <t>Claymore</t>
+  </si>
+  <si>
+    <t>BattleAxe</t>
+  </si>
+  <si>
+    <t>Arena Knuckles</t>
+  </si>
+  <si>
+    <t>Pilot REF -3</t>
+  </si>
+  <si>
+    <t>Pilot REF +3</t>
+  </si>
+  <si>
+    <t>(Tonnage/10) +1</t>
+  </si>
+  <si>
+    <t>(Tonnage/10) +2</t>
+  </si>
+  <si>
+    <t>(Tonnage/10) +3</t>
+  </si>
+  <si>
+    <t>Club (improvised)</t>
+  </si>
+  <si>
+    <t>Standard Melee</t>
+  </si>
+  <si>
+    <t>Battle Flail</t>
+  </si>
+  <si>
+    <t>Pilot REF -2</t>
+  </si>
+  <si>
+    <t>Pilot REF -4</t>
+  </si>
+  <si>
+    <t>(Tonnage/10) +4</t>
   </si>
 </sst>
 </file>
@@ -368,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -395,9 +455,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -737,7 +794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFC43064-AB08-4B2D-9CB9-2FA6A7A44140}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" bestFit="1" customWidth="1"/>
@@ -745,6 +802,7 @@
     <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1837,19 +1895,19 @@
       <c r="A39" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B39" s="12" t="s">
         <v>46</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D39" s="12" t="s">
+      <c r="D39" s="4" t="s">
         <v>16</v>
       </c>
       <c r="E39" s="5">
         <v>3</v>
       </c>
-      <c r="F39" s="12">
+      <c r="F39" s="4">
         <v>0</v>
       </c>
       <c r="G39" s="4">
@@ -2049,7 +2107,9 @@
       <c r="D46" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="4"/>
+      <c r="E46" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -2066,9 +2126,11 @@
         <v>34</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="E47" s="8"/>
+        <v>87</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>24</v>
+      </c>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
@@ -2087,14 +2149,278 @@
       <c r="D48" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E48" s="8"/>
+      <c r="E48" s="8" t="s">
+        <v>24</v>
+      </c>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="8"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1"/>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E49" s="10">
+        <v>0</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E50" s="10">
+        <v>0</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E51" s="10">
+        <v>0</v>
+      </c>
+      <c r="F51" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E52" s="10">
+        <v>0</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E53" s="10">
+        <v>0</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E54" s="10">
+        <v>0</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I54" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E55" s="10">
+        <v>0</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="G55" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E56" s="10">
+        <v>0</v>
+      </c>
+      <c r="F56" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E57" s="10">
+        <v>0</v>
+      </c>
+      <c r="F57" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="1"/>
+      <c r="B58" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Fixed the machine monitor semantics test to properly test the semantics of machine monitors, rather than just testing that the monitor values are correct. This involved adding assertions to check that the correct monitors are active based on the machine's current state, and that the correct effects are applied when monitors are active. Additionally, I updated the test data to better reflect realistic scenarios for machine monitor activation and effects.
</commit_message>
<xml_diff>
--- a/docs/Mech-Weapons.xlsx
+++ b/docs/Mech-Weapons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FoundryData-Dev\Data\systems\mwd\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85488DC7-86ED-4D29-BB1C-079C71C0743B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF8D95C-22E4-4B96-9535-7587414E6B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="-4995" windowWidth="16440" windowHeight="28320" xr2:uid="{E1E4146D-AA47-4F02-8EE5-13D857F0DD65}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="110">
   <si>
     <t>Weapon</t>
   </si>
@@ -355,6 +355,18 @@
   </si>
   <si>
     <t>10</t>
+  </si>
+  <si>
+    <t>-8</t>
+  </si>
+  <si>
+    <t>-4</t>
+  </si>
+  <si>
+    <t>-6</t>
+  </si>
+  <si>
+    <t>6</t>
   </si>
 </sst>
 </file>
@@ -974,8 +986,8 @@
       <c r="D5" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E5" s="9">
-        <v>1</v>
+      <c r="E5" s="9" t="s">
+        <v>24</v>
       </c>
       <c r="F5" s="8">
         <v>-5</v>
@@ -1076,14 +1088,14 @@
       <c r="F8" s="4">
         <v>-5</v>
       </c>
-      <c r="G8" s="4">
-        <v>-1</v>
-      </c>
-      <c r="H8" s="4">
-        <v>-4</v>
+      <c r="G8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>3</v>
+        <v>107</v>
       </c>
       <c r="J8" s="16">
         <v>125000</v>
@@ -1105,17 +1117,17 @@
       <c r="E9" s="5">
         <v>0</v>
       </c>
-      <c r="F9" s="4">
-        <v>-5</v>
-      </c>
-      <c r="G9" s="4">
-        <v>-1</v>
-      </c>
-      <c r="H9" s="4">
-        <v>-4</v>
+      <c r="F9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>60</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>3</v>
+        <v>108</v>
       </c>
       <c r="J9" s="16">
         <v>200000</v>
@@ -1131,14 +1143,24 @@
       <c r="C10" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="5"/>
+      <c r="D10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="F10" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="14"/>
+        <v>51</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>51</v>
+      </c>
       <c r="J10" s="16">
         <v>250000</v>
       </c>
@@ -1153,14 +1175,24 @@
       <c r="C11" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="F11" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="14"/>
+      <c r="G11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>106</v>
+      </c>
       <c r="J11" s="16">
         <v>275000</v>
       </c>
@@ -1181,14 +1213,14 @@
       <c r="E12" s="9">
         <v>1</v>
       </c>
-      <c r="F12" s="8">
-        <v>0</v>
-      </c>
-      <c r="G12" s="8">
-        <v>-1</v>
-      </c>
-      <c r="H12" s="8">
-        <v>-4</v>
+      <c r="F12" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>102</v>
       </c>
       <c r="I12" s="13" t="s">
         <v>3</v>
@@ -1207,12 +1239,24 @@
       <c r="C13" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="8"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="13"/>
+      <c r="D13" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="13" t="s">
+        <v>3</v>
+      </c>
       <c r="J13" s="18">
         <v>320000</v>
       </c>
@@ -1227,12 +1271,24 @@
       <c r="C14" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="13"/>
+      <c r="D14" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>3</v>
+      </c>
       <c r="J14" s="18">
         <v>400000</v>
       </c>
@@ -1253,11 +1309,11 @@
       <c r="E15" s="5">
         <v>2</v>
       </c>
-      <c r="F15" s="4">
-        <v>2</v>
-      </c>
-      <c r="G15" s="4">
-        <v>-1</v>
+      <c r="F15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>3</v>
@@ -1279,12 +1335,24 @@
       <c r="C16" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="14"/>
+      <c r="D16" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>3</v>
+      </c>
       <c r="J16" s="16">
         <v>480000</v>
       </c>
@@ -1299,12 +1367,24 @@
       <c r="C17" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="14"/>
+      <c r="D17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>3</v>
+      </c>
       <c r="J17" s="16">
         <v>600000</v>
       </c>
@@ -1325,10 +1405,18 @@
       <c r="E18" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="13"/>
+      <c r="F18" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>102</v>
+      </c>
       <c r="J18" s="18">
         <v>300000</v>
       </c>
@@ -1349,10 +1437,18 @@
       <c r="E19" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="13"/>
+      <c r="F19" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="I19" s="13" t="s">
+        <v>102</v>
+      </c>
       <c r="J19" s="18">
         <v>500000</v>
       </c>
@@ -1373,10 +1469,18 @@
       <c r="E20" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="13"/>
+      <c r="F20" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>102</v>
+      </c>
       <c r="J20" s="18">
         <v>275000</v>
       </c>
@@ -1845,11 +1949,11 @@
       <c r="E35" s="9">
         <v>2</v>
       </c>
-      <c r="F35" s="8">
-        <v>2</v>
-      </c>
-      <c r="G35" s="8">
-        <v>0</v>
+      <c r="F35" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="H35" s="8" t="s">
         <v>3</v>
@@ -1909,14 +2013,14 @@
       <c r="E37" s="5">
         <v>2</v>
       </c>
-      <c r="F37" s="4">
-        <v>5</v>
-      </c>
-      <c r="G37" s="4">
-        <v>2</v>
-      </c>
-      <c r="H37" s="4">
-        <v>0</v>
+      <c r="F37" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>3</v>
@@ -1941,11 +2045,11 @@
       <c r="E38" s="5">
         <v>2</v>
       </c>
-      <c r="F38" s="4">
-        <v>5</v>
-      </c>
-      <c r="G38" s="4">
-        <v>2</v>
+      <c r="F38" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>3</v>
@@ -1970,17 +2074,17 @@
       <c r="D39" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E39" s="5">
-        <v>2</v>
-      </c>
-      <c r="F39" s="4">
-        <v>2</v>
-      </c>
-      <c r="G39" s="4">
-        <v>-1</v>
+      <c r="E39" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>3</v>
@@ -2037,17 +2141,17 @@
       <c r="E41" s="9">
         <v>3</v>
       </c>
-      <c r="F41" s="8">
-        <v>5</v>
+      <c r="F41" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="G41" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H41" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="H41" s="8">
-        <v>-2</v>
-      </c>
-      <c r="I41" s="13">
-        <v>-1</v>
+      <c r="I41" s="13" t="s">
+        <v>24</v>
       </c>
       <c r="J41" s="18">
         <v>200000</v>
@@ -2069,14 +2173,14 @@
       <c r="E42" s="9">
         <v>3</v>
       </c>
-      <c r="F42" s="8">
-        <v>5</v>
-      </c>
-      <c r="G42" s="8">
-        <v>0</v>
+      <c r="F42" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="I42" s="13" t="s">
         <v>3</v>
@@ -2101,17 +2205,17 @@
       <c r="E43" s="9">
         <v>4</v>
       </c>
-      <c r="F43" s="8">
-        <v>4</v>
+      <c r="F43" s="8" t="s">
+        <v>109</v>
       </c>
       <c r="G43" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H43" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H43" s="8" t="s">
-        <v>51</v>
-      </c>
       <c r="I43" s="13" t="s">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="J43" s="18">
         <v>275000</v>

</xml_diff>